<commit_message>
feat(v2): universal file parsing engine, database sequence & Cartesian fixes, batch sales/invoices import, and cloud deployment config
</commit_message>
<xml_diff>
--- a/exports/sales_current_month.xlsx
+++ b/exports/sales_current_month.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>Accounting Master Report - Current Month Sales (Generated: 9/2/2026, 9:57:37 PM)</t>
+    <t>Accounting Master Report - Current Month Sales (Generated: 9/12/2026, 10:15:30 AM)</t>
   </si>
   <si>
     <t>Sale ID</t>
@@ -462,7 +462,7 @@
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="11" width="84" customWidth="1"/>
+    <col min="1" max="11" width="86" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>